<commit_message>
Update test scenario and added test case of login page
</commit_message>
<xml_diff>
--- a/Project-2/TestScenario_SauceDemo.xlsx
+++ b/Project-2/TestScenario_SauceDemo.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADARSH J. MISHRA\OneDrive\GitHub-Backup\Manual-Testing-Projects\Project-2\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/d09b73bd954f8bef/GitHub-Backup/Manual-Testing-Projects/Project-2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8134D4F3-0D94-4D59-BC84-9586F3F5E83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="14" documentId="13_ncr:1_{8134D4F3-0D94-4D59-BC84-9586F3F5E83E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{23D02E85-907C-452F-99CE-A589F1DA7E82}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{AE7A96EB-CAF4-4974-9235-C6F64EFA36B0}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="77">
   <si>
     <t>Login Module</t>
   </si>
@@ -60,9 +60,6 @@
     <t>Login</t>
   </si>
   <si>
-    <t>Verify login with valid username and password</t>
-  </si>
-  <si>
     <t>High</t>
   </si>
   <si>
@@ -87,24 +84,12 @@
     <t>TS_05</t>
   </si>
   <si>
-    <t>Verify login with invalid username</t>
-  </si>
-  <si>
-    <t>Verify login with invalid password</t>
-  </si>
-  <si>
     <t>TS_06</t>
   </si>
   <si>
     <t>TS_07</t>
   </si>
   <si>
-    <t>Verify login with empty password</t>
-  </si>
-  <si>
-    <t>Verify login with empty username</t>
-  </si>
-  <si>
     <t>TS_08</t>
   </si>
   <si>
@@ -120,9 +105,6 @@
     <t>Verify login of all accepted users with invalid password</t>
   </si>
   <si>
-    <t>Verify login with invalid username and password</t>
-  </si>
-  <si>
     <t>TS_11</t>
   </si>
   <si>
@@ -273,25 +255,19 @@
     <t>Verify product price</t>
   </si>
   <si>
-    <t>TS_32</t>
-  </si>
-  <si>
-    <t>TS_33</t>
-  </si>
-  <si>
     <t>Verify order confirmation after finish</t>
   </si>
   <si>
-    <t>TS_34</t>
-  </si>
-  <si>
     <t>Verify user can go directly product page after back to home button on order confirmation page</t>
   </si>
   <si>
-    <t>TS_35</t>
-  </si>
-  <si>
     <t>Verify user can go login page after clicking logout</t>
+  </si>
+  <si>
+    <t>Verify login with valid credentials</t>
+  </si>
+  <si>
+    <t>Verify login with invalid credentials</t>
   </si>
 </sst>
 </file>
@@ -445,7 +421,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -454,6 +430,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -473,12 +452,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -802,7 +775,7 @@
   <sheetPr>
     <tabColor rgb="FF7030A0"/>
   </sheetPr>
-  <dimension ref="A1:D15"/>
+  <dimension ref="A1:D11"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13.33203125" customWidth="1"/>
@@ -812,18 +785,18 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
+      <c r="A1" s="5" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="6"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="4" spans="1:4" ht="18" x14ac:dyDescent="0.3">
       <c r="A4" s="2" t="s">
@@ -847,156 +820,101 @@
         <v>6</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>7</v>
+        <v>75</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>27</v>
+        <v>76</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="3" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" s="1" t="s">
         <v>12</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="3" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="3" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="3" t="s">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A12" s="3" t="s">
-        <v>22</v>
-      </c>
-      <c r="B12" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A13" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B13" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C13" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="D13" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A14" s="3" t="s">
-        <v>25</v>
-      </c>
-      <c r="B14" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C14" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D14" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>29</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D2"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1016,135 +934,136 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>30</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="6"/>
+      <c r="A1" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>31</v>
+        <v>17</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>34</v>
+        <v>18</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>37</v>
+        <v>20</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>39</v>
+        <v>22</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>38</v>
+        <v>32</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>40</v>
+        <v>34</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>41</v>
+        <v>35</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>43</v>
+        <v>28</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>32</v>
+        <v>26</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A11" s="10" t="s">
-        <v>46</v>
-      </c>
-      <c r="B11" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C11" s="10" t="s">
-        <v>84</v>
-      </c>
-      <c r="D11" s="10" t="s">
-        <v>8</v>
+      <c r="A11" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="B11" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:D2"/>
   </mergeCells>
+  <phoneticPr fontId="4" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -1161,115 +1080,115 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>45</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="6"/>
+      <c r="A1" s="5" t="s">
+        <v>39</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>49</v>
+        <v>33</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>48</v>
+        <v>42</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>51</v>
+        <v>36</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>50</v>
+        <v>44</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>52</v>
+        <v>46</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>55</v>
+        <v>40</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>54</v>
+        <v>48</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>57</v>
+        <v>43</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>56</v>
+        <v>50</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>60</v>
+        <v>45</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
   </sheetData>
@@ -1296,185 +1215,185 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="4" t="s">
-        <v>59</v>
-      </c>
-      <c r="B1" s="5"/>
-      <c r="C1" s="5"/>
-      <c r="D1" s="6"/>
+      <c r="A1" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="7"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="9"/>
+      <c r="A2" s="8"/>
+      <c r="B2" s="9"/>
+      <c r="C2" s="9"/>
+      <c r="D2" s="10"/>
     </row>
     <row r="4" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="11" t="s">
+      <c r="C4" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="D4" s="11" t="s">
+      <c r="D4" s="4" t="s">
         <v>4</v>
       </c>
     </row>
     <row r="5" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
-        <v>65</v>
+        <v>49</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>64</v>
+        <v>58</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="7" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
-        <v>67</v>
+        <v>51</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>66</v>
+        <v>60</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="8" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
-        <v>69</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>68</v>
+        <v>62</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="10" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
-        <v>73</v>
+        <v>59</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>72</v>
+        <v>66</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
-        <v>75</v>
+        <v>61</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>74</v>
+        <v>68</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="12" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="B12" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C12" s="10" t="s">
-        <v>76</v>
-      </c>
-      <c r="D12" s="10" t="s">
-        <v>8</v>
+        <v>63</v>
+      </c>
+      <c r="B12" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="13" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
-        <v>79</v>
-      </c>
-      <c r="B13" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C13" s="10" t="s">
-        <v>77</v>
-      </c>
-      <c r="D13" s="10" t="s">
-        <v>8</v>
+        <v>65</v>
+      </c>
+      <c r="B13" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="D13" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="14" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B14" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C14" s="10" t="s">
-        <v>80</v>
-      </c>
-      <c r="D14" s="10" t="s">
-        <v>8</v>
+        <v>67</v>
+      </c>
+      <c r="B14" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="D14" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
     <row r="15" spans="1:4" ht="15.6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B15" s="10" t="s">
-        <v>61</v>
-      </c>
-      <c r="C15" s="10" t="s">
-        <v>82</v>
-      </c>
-      <c r="D15" s="10" t="s">
-        <v>8</v>
+        <v>69</v>
+      </c>
+      <c r="B15" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="D15" s="1" t="s">
+        <v>7</v>
       </c>
     </row>
   </sheetData>

</xml_diff>